<commit_message>
Database - Refresh Test Data - 26.10.2024
</commit_message>
<xml_diff>
--- a/java22 database design/Java22 QPhan Database Design.xlsx
+++ b/java22 database design/Java22 QPhan Database Design.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qphan\Desktop\bkit\course - webapp\java22\3. Database\java22 database design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AE5FF7E-357E-4DDE-84AB-7D058AB496AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB07CED2-C537-40AD-A8C7-EE9852DAE1FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" tabRatio="901" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38340" yWindow="-1770" windowWidth="29265" windowHeight="19515" tabRatio="901" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="B1. Mô hình quan niệm" sheetId="1" r:id="rId1"/>
@@ -627,7 +627,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1146" uniqueCount="553">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1148" uniqueCount="565">
   <si>
     <t>NhanVien</t>
   </si>
@@ -2300,12 +2300,48 @@
   <si>
     <t>[red, yelllow, blue, green, orange]</t>
   </si>
+  <si>
+    <t>sha…</t>
+  </si>
+  <si>
+    <t>bcrypt</t>
+  </si>
+  <si>
+    <t>c1@gmail.com</t>
+  </si>
+  <si>
+    <t>c2@gmail.com</t>
+  </si>
+  <si>
+    <t>c3@gmail.com</t>
+  </si>
+  <si>
+    <t>c4@gmail.com</t>
+  </si>
+  <si>
+    <t>c5@gmail.com</t>
+  </si>
+  <si>
+    <t>c6@gmail.com</t>
+  </si>
+  <si>
+    <t>c7@gmail.com</t>
+  </si>
+  <si>
+    <t>c8@gmail.com</t>
+  </si>
+  <si>
+    <t>c9@gmail.com</t>
+  </si>
+  <si>
+    <t>c10@gmail.com</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="28" x14ac:knownFonts="1">
+  <fonts count="29" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2507,6 +2543,14 @@
       <name val="Tahoma"/>
       <charset val="1"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -2597,10 +2641,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2816,8 +2861,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -9329,6 +9384,9 @@
       <c r="C75" s="28" t="s">
         <v>509</v>
       </c>
+      <c r="F75" s="27" t="s">
+        <v>553</v>
+      </c>
     </row>
     <row r="76" spans="2:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B76" s="28">
@@ -9336,6 +9394,9 @@
       </c>
       <c r="C76" s="28" t="s">
         <v>510</v>
+      </c>
+      <c r="F76" s="27" t="s">
+        <v>554</v>
       </c>
     </row>
     <row r="77" spans="2:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -9375,7 +9436,7 @@
         <v>511</v>
       </c>
       <c r="D80" s="29" t="s">
-        <v>180</v>
+        <v>555</v>
       </c>
       <c r="E80" s="28" t="s">
         <v>200</v>
@@ -9394,8 +9455,8 @@
       <c r="C81" s="28" t="s">
         <v>512</v>
       </c>
-      <c r="D81" s="28" t="s">
-        <v>181</v>
+      <c r="D81" s="75" t="s">
+        <v>556</v>
       </c>
       <c r="E81" s="28" t="s">
         <v>201</v>
@@ -9414,8 +9475,8 @@
       <c r="C82" s="28" t="s">
         <v>513</v>
       </c>
-      <c r="D82" s="28" t="s">
-        <v>182</v>
+      <c r="D82" s="29" t="s">
+        <v>557</v>
       </c>
       <c r="E82" s="28" t="s">
         <v>202</v>
@@ -9434,8 +9495,8 @@
       <c r="C83" s="28" t="s">
         <v>514</v>
       </c>
-      <c r="D83" s="28" t="s">
-        <v>183</v>
+      <c r="D83" s="76" t="s">
+        <v>558</v>
       </c>
       <c r="E83" s="28" t="s">
         <v>203</v>
@@ -9454,8 +9515,8 @@
       <c r="C84" s="28" t="s">
         <v>515</v>
       </c>
-      <c r="D84" s="28" t="s">
-        <v>184</v>
+      <c r="D84" s="29" t="s">
+        <v>559</v>
       </c>
       <c r="E84" s="28" t="s">
         <v>204</v>
@@ -9474,8 +9535,8 @@
       <c r="C85" s="28" t="s">
         <v>516</v>
       </c>
-      <c r="D85" s="28" t="s">
-        <v>185</v>
+      <c r="D85" s="76" t="s">
+        <v>560</v>
       </c>
       <c r="E85" s="28" t="s">
         <v>205</v>
@@ -9494,8 +9555,8 @@
       <c r="C86" s="28" t="s">
         <v>517</v>
       </c>
-      <c r="D86" s="28" t="s">
-        <v>186</v>
+      <c r="D86" s="29" t="s">
+        <v>561</v>
       </c>
       <c r="E86" s="28" t="s">
         <v>206</v>
@@ -9514,8 +9575,8 @@
       <c r="C87" s="28" t="s">
         <v>518</v>
       </c>
-      <c r="D87" s="28" t="s">
-        <v>187</v>
+      <c r="D87" s="76" t="s">
+        <v>562</v>
       </c>
       <c r="E87" s="28" t="s">
         <v>207</v>
@@ -9534,8 +9595,8 @@
       <c r="C88" s="28" t="s">
         <v>519</v>
       </c>
-      <c r="D88" s="28" t="s">
-        <v>188</v>
+      <c r="D88" s="29" t="s">
+        <v>563</v>
       </c>
       <c r="E88" s="28" t="s">
         <v>208</v>
@@ -9554,8 +9615,8 @@
       <c r="C89" s="28" t="s">
         <v>520</v>
       </c>
-      <c r="D89" s="28" t="s">
-        <v>189</v>
+      <c r="D89" s="77" t="s">
+        <v>564</v>
       </c>
       <c r="E89" s="28" t="s">
         <v>209</v>
@@ -11045,8 +11106,14 @@
     <mergeCell ref="C161:D161"/>
   </mergeCells>
   <phoneticPr fontId="16" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="D83" r:id="rId1" xr:uid="{06FB0EAA-DB26-4E19-8EC1-C6A4ABFA945E}"/>
+    <hyperlink ref="D85" r:id="rId2" xr:uid="{8C283B2C-EDF8-4F34-9AB0-5B631ED14338}"/>
+    <hyperlink ref="D87" r:id="rId3" xr:uid="{A6FC5845-C6DA-4EA8-8A5A-F571CF4AF45D}"/>
+    <hyperlink ref="D89" r:id="rId4" xr:uid="{7364BA95-4D85-46B9-8EC3-51D7C930A631}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
+  <legacyDrawing r:id="rId5"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Finish refresh test data - 27.10.2024
</commit_message>
<xml_diff>
--- a/java22 database design/Java22 QPhan Database Design.xlsx
+++ b/java22 database design/Java22 QPhan Database Design.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qphan\Desktop\bkit\course - webapp\java22\3. Database\java22 database design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB07CED2-C537-40AD-A8C7-EE9852DAE1FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD2A3297-426B-4E82-86C0-6E3812248BEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38340" yWindow="-1770" windowWidth="29265" windowHeight="19515" tabRatio="901" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-2025" windowWidth="38640" windowHeight="21240" tabRatio="901" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="B1. Mô hình quan niệm" sheetId="1" r:id="rId1"/>
@@ -627,7 +627,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1148" uniqueCount="565">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1148" uniqueCount="566">
   <si>
     <t>NhanVien</t>
   </si>
@@ -2335,6 +2335,9 @@
   </si>
   <si>
     <t>c10@gmail.com</t>
+  </si>
+  <si>
+    <t>-- 4. Đơn hàng từ 11 - 12 --&gt; Hủy đơn hàng (trạng thái 1 và 7)</t>
   </si>
 </sst>
 </file>
@@ -2645,7 +2648,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2834,6 +2837,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -2859,15 +2868,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -5600,16 +5600,16 @@
     </row>
     <row r="72" spans="2:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="73" spans="2:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C73" s="72" t="s">
+      <c r="C73" s="74" t="s">
         <v>277</v>
       </c>
-      <c r="D73" s="72"/>
-      <c r="E73" s="72"/>
+      <c r="D73" s="74"/>
+      <c r="E73" s="74"/>
     </row>
     <row r="74" spans="2:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C74" s="72"/>
-      <c r="D74" s="72"/>
-      <c r="E74" s="72"/>
+      <c r="C74" s="74"/>
+      <c r="D74" s="74"/>
+      <c r="E74" s="74"/>
     </row>
     <row r="75" spans="2:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="76" spans="2:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -5633,14 +5633,14 @@
     </row>
     <row r="78" spans="2:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="79" spans="2:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C79" s="72" t="s">
+      <c r="C79" s="74" t="s">
         <v>277</v>
       </c>
-      <c r="D79" s="72"/>
+      <c r="D79" s="74"/>
     </row>
     <row r="80" spans="2:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C80" s="72"/>
-      <c r="D80" s="72"/>
+      <c r="C80" s="74"/>
+      <c r="D80" s="74"/>
     </row>
     <row r="81" spans="2:7" ht="21.95" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="82" spans="2:7" ht="21.95" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -5675,30 +5675,30 @@
       </c>
     </row>
     <row r="86" spans="2:7" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C86" s="73" t="s">
+      <c r="C86" s="75" t="s">
         <v>283</v>
       </c>
-      <c r="D86" s="72"/>
-      <c r="E86" s="72"/>
-      <c r="F86" s="72"/>
+      <c r="D86" s="74"/>
+      <c r="E86" s="74"/>
+      <c r="F86" s="74"/>
     </row>
     <row r="87" spans="2:7" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C87" s="72"/>
-      <c r="D87" s="72"/>
-      <c r="E87" s="72"/>
-      <c r="F87" s="72"/>
+      <c r="C87" s="74"/>
+      <c r="D87" s="74"/>
+      <c r="E87" s="74"/>
+      <c r="F87" s="74"/>
     </row>
     <row r="88" spans="2:7" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C88" s="72"/>
-      <c r="D88" s="72"/>
-      <c r="E88" s="72"/>
-      <c r="F88" s="72"/>
+      <c r="C88" s="74"/>
+      <c r="D88" s="74"/>
+      <c r="E88" s="74"/>
+      <c r="F88" s="74"/>
     </row>
     <row r="89" spans="2:7" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C89" s="72"/>
-      <c r="D89" s="72"/>
-      <c r="E89" s="72"/>
-      <c r="F89" s="72"/>
+      <c r="C89" s="74"/>
+      <c r="D89" s="74"/>
+      <c r="E89" s="74"/>
+      <c r="F89" s="74"/>
     </row>
     <row r="90" spans="2:7" ht="21.95" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="91" spans="2:7" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -5715,18 +5715,18 @@
       </c>
     </row>
     <row r="93" spans="2:7" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B93" s="74" t="s">
+      <c r="B93" s="76" t="s">
         <v>280</v>
       </c>
-      <c r="C93" s="74"/>
+      <c r="C93" s="76"/>
     </row>
     <row r="94" spans="2:7" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B94" s="72"/>
-      <c r="C94" s="72"/>
+      <c r="B94" s="74"/>
+      <c r="C94" s="74"/>
     </row>
     <row r="95" spans="2:7" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B95" s="72"/>
-      <c r="C95" s="72"/>
+      <c r="B95" s="74"/>
+      <c r="C95" s="74"/>
     </row>
     <row r="96" spans="2:7" ht="21.95" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="97" spans="2:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -5749,11 +5749,11 @@
       </c>
     </row>
     <row r="99" spans="2:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B99" s="71" t="s">
+      <c r="B99" s="73" t="s">
         <v>281</v>
       </c>
-      <c r="C99" s="71"/>
-      <c r="D99" s="71"/>
+      <c r="C99" s="73"/>
+      <c r="D99" s="73"/>
       <c r="F99" s="14" t="s">
         <v>112</v>
       </c>
@@ -5768,14 +5768,14 @@
       </c>
     </row>
     <row r="100" spans="2:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B100" s="71"/>
-      <c r="C100" s="71"/>
-      <c r="D100" s="71"/>
+      <c r="B100" s="73"/>
+      <c r="C100" s="73"/>
+      <c r="D100" s="73"/>
     </row>
     <row r="101" spans="2:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B101" s="71"/>
-      <c r="C101" s="71"/>
-      <c r="D101" s="71"/>
+      <c r="B101" s="73"/>
+      <c r="C101" s="73"/>
+      <c r="D101" s="73"/>
       <c r="F101" s="31" t="s">
         <v>297</v>
       </c>
@@ -7464,15 +7464,15 @@
       <c r="K16" s="24"/>
     </row>
     <row r="17" spans="2:11" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="66" t="s">
+      <c r="B17" s="68" t="s">
         <v>45</v>
       </c>
-      <c r="C17" s="66"/>
-      <c r="D17" s="66"/>
-      <c r="E17" s="66"/>
-      <c r="G17" s="68"/>
-      <c r="H17" s="68"/>
-      <c r="I17" s="68"/>
+      <c r="C17" s="68"/>
+      <c r="D17" s="68"/>
+      <c r="E17" s="68"/>
+      <c r="G17" s="70"/>
+      <c r="H17" s="70"/>
+      <c r="I17" s="70"/>
     </row>
     <row r="18" spans="2:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="10" t="s">
@@ -7484,12 +7484,12 @@
       <c r="I18" s="19"/>
     </row>
     <row r="19" spans="2:11" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="66" t="s">
+      <c r="B19" s="68" t="s">
         <v>46</v>
       </c>
-      <c r="C19" s="67"/>
-      <c r="D19" s="67"/>
-      <c r="E19" s="67"/>
+      <c r="C19" s="69"/>
+      <c r="D19" s="69"/>
+      <c r="E19" s="69"/>
       <c r="J19" s="17"/>
       <c r="K19" s="17"/>
     </row>
@@ -7501,12 +7501,12 @@
       <c r="K20" s="17"/>
     </row>
     <row r="21" spans="2:11" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="66" t="s">
+      <c r="B21" s="68" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="69"/>
-      <c r="D21" s="69"/>
-      <c r="E21" s="69"/>
+      <c r="C21" s="71"/>
+      <c r="D21" s="71"/>
+      <c r="E21" s="71"/>
       <c r="J21" s="17"/>
       <c r="K21" s="17"/>
     </row>
@@ -7521,32 +7521,32 @@
       <c r="K22" s="20"/>
     </row>
     <row r="23" spans="2:11" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="66" t="s">
+      <c r="B23" s="68" t="s">
         <v>50</v>
       </c>
-      <c r="C23" s="66"/>
-      <c r="D23" s="66"/>
-      <c r="E23" s="66"/>
+      <c r="C23" s="68"/>
+      <c r="D23" s="68"/>
+      <c r="E23" s="68"/>
       <c r="J23" s="7"/>
       <c r="K23" s="7"/>
     </row>
     <row r="24" spans="2:11" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="66" t="s">
+      <c r="B24" s="68" t="s">
         <v>338</v>
       </c>
-      <c r="C24" s="67"/>
-      <c r="D24" s="67"/>
-      <c r="E24" s="67"/>
+      <c r="C24" s="69"/>
+      <c r="D24" s="69"/>
+      <c r="E24" s="69"/>
       <c r="J24" s="7"/>
       <c r="K24" s="7"/>
     </row>
     <row r="25" spans="2:11" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="66" t="s">
+      <c r="B25" s="68" t="s">
         <v>51</v>
       </c>
-      <c r="C25" s="67"/>
-      <c r="D25" s="67"/>
-      <c r="E25" s="67"/>
+      <c r="C25" s="69"/>
+      <c r="D25" s="69"/>
+      <c r="E25" s="69"/>
       <c r="F25" s="15"/>
       <c r="G25" s="15"/>
       <c r="H25" s="4"/>
@@ -8243,15 +8243,15 @@
       </c>
     </row>
     <row r="17" spans="4:18" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D17" s="66" t="s">
+      <c r="D17" s="68" t="s">
         <v>45</v>
       </c>
-      <c r="E17" s="66"/>
-      <c r="F17" s="66"/>
-      <c r="G17" s="66"/>
-      <c r="H17" s="66"/>
-      <c r="I17" s="66"/>
-      <c r="J17" s="66"/>
+      <c r="E17" s="68"/>
+      <c r="F17" s="68"/>
+      <c r="G17" s="68"/>
+      <c r="H17" s="68"/>
+      <c r="I17" s="68"/>
+      <c r="J17" s="68"/>
       <c r="K17" s="37"/>
       <c r="L17" s="37"/>
       <c r="M17" s="37"/>
@@ -8286,15 +8286,15 @@
       </c>
     </row>
     <row r="19" spans="4:18" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D19" s="66" t="s">
+      <c r="D19" s="68" t="s">
         <v>46</v>
       </c>
-      <c r="E19" s="67"/>
-      <c r="F19" s="67"/>
-      <c r="G19" s="67"/>
-      <c r="H19" s="67"/>
-      <c r="I19" s="67"/>
-      <c r="J19" s="67"/>
+      <c r="E19" s="69"/>
+      <c r="F19" s="69"/>
+      <c r="G19" s="69"/>
+      <c r="H19" s="69"/>
+      <c r="I19" s="69"/>
+      <c r="J19" s="69"/>
       <c r="N19" s="17"/>
       <c r="O19" s="17">
         <v>3</v>
@@ -8322,15 +8322,15 @@
       </c>
     </row>
     <row r="21" spans="4:18" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D21" s="66" t="s">
+      <c r="D21" s="68" t="s">
         <v>48</v>
       </c>
-      <c r="E21" s="69"/>
-      <c r="F21" s="69"/>
-      <c r="G21" s="69"/>
-      <c r="H21" s="69"/>
-      <c r="I21" s="69"/>
-      <c r="J21" s="69"/>
+      <c r="E21" s="71"/>
+      <c r="F21" s="71"/>
+      <c r="G21" s="71"/>
+      <c r="H21" s="71"/>
+      <c r="I21" s="71"/>
+      <c r="J21" s="71"/>
       <c r="N21" s="17"/>
       <c r="O21" s="1">
         <v>5</v>
@@ -8364,15 +8364,15 @@
       </c>
     </row>
     <row r="23" spans="4:18" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D23" s="66" t="s">
+      <c r="D23" s="68" t="s">
         <v>50</v>
       </c>
-      <c r="E23" s="66"/>
-      <c r="F23" s="66"/>
-      <c r="G23" s="66"/>
-      <c r="H23" s="66"/>
-      <c r="I23" s="66"/>
-      <c r="J23" s="66"/>
+      <c r="E23" s="68"/>
+      <c r="F23" s="68"/>
+      <c r="G23" s="68"/>
+      <c r="H23" s="68"/>
+      <c r="I23" s="68"/>
+      <c r="J23" s="68"/>
       <c r="N23" s="7"/>
       <c r="O23" s="17">
         <v>7</v>
@@ -8385,15 +8385,15 @@
       </c>
     </row>
     <row r="24" spans="4:18" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D24" s="66" t="s">
+      <c r="D24" s="68" t="s">
         <v>338</v>
       </c>
-      <c r="E24" s="67"/>
-      <c r="F24" s="67"/>
-      <c r="G24" s="67"/>
-      <c r="H24" s="67"/>
-      <c r="I24" s="67"/>
-      <c r="J24" s="67"/>
+      <c r="E24" s="69"/>
+      <c r="F24" s="69"/>
+      <c r="G24" s="69"/>
+      <c r="H24" s="69"/>
+      <c r="I24" s="69"/>
+      <c r="J24" s="69"/>
       <c r="N24" s="7"/>
       <c r="O24" s="17">
         <v>8</v>
@@ -8406,15 +8406,15 @@
       </c>
     </row>
     <row r="25" spans="4:18" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D25" s="66" t="s">
+      <c r="D25" s="68" t="s">
         <v>51</v>
       </c>
-      <c r="E25" s="67"/>
-      <c r="F25" s="67"/>
-      <c r="G25" s="67"/>
-      <c r="H25" s="67"/>
-      <c r="I25" s="67"/>
-      <c r="J25" s="67"/>
+      <c r="E25" s="69"/>
+      <c r="F25" s="69"/>
+      <c r="G25" s="69"/>
+      <c r="H25" s="69"/>
+      <c r="I25" s="69"/>
+      <c r="J25" s="69"/>
       <c r="K25" s="15"/>
       <c r="L25" s="4"/>
       <c r="P25" s="15"/>
@@ -9330,30 +9330,30 @@
       </c>
     </row>
     <row r="67" spans="2:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C67" s="70" t="s">
+      <c r="C67" s="72" t="s">
         <v>507</v>
       </c>
-      <c r="D67" s="68"/>
-      <c r="E67" s="68"/>
-      <c r="F67" s="68"/>
+      <c r="D67" s="70"/>
+      <c r="E67" s="70"/>
+      <c r="F67" s="70"/>
     </row>
     <row r="68" spans="2:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C68" s="68"/>
-      <c r="D68" s="68"/>
-      <c r="E68" s="68"/>
-      <c r="F68" s="68"/>
+      <c r="C68" s="70"/>
+      <c r="D68" s="70"/>
+      <c r="E68" s="70"/>
+      <c r="F68" s="70"/>
     </row>
     <row r="69" spans="2:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C69" s="68"/>
-      <c r="D69" s="68"/>
-      <c r="E69" s="68"/>
-      <c r="F69" s="68"/>
+      <c r="C69" s="70"/>
+      <c r="D69" s="70"/>
+      <c r="E69" s="70"/>
+      <c r="F69" s="70"/>
     </row>
     <row r="70" spans="2:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C70" s="68"/>
-      <c r="D70" s="68"/>
-      <c r="E70" s="68"/>
-      <c r="F70" s="68"/>
+      <c r="C70" s="70"/>
+      <c r="D70" s="70"/>
+      <c r="E70" s="70"/>
+      <c r="F70" s="70"/>
     </row>
     <row r="71" spans="2:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="72" spans="2:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -9455,7 +9455,7 @@
       <c r="C81" s="28" t="s">
         <v>512</v>
       </c>
-      <c r="D81" s="75" t="s">
+      <c r="D81" s="27" t="s">
         <v>556</v>
       </c>
       <c r="E81" s="28" t="s">
@@ -9495,7 +9495,7 @@
       <c r="C83" s="28" t="s">
         <v>514</v>
       </c>
-      <c r="D83" s="76" t="s">
+      <c r="D83" s="66" t="s">
         <v>558</v>
       </c>
       <c r="E83" s="28" t="s">
@@ -9535,7 +9535,7 @@
       <c r="C85" s="28" t="s">
         <v>516</v>
       </c>
-      <c r="D85" s="76" t="s">
+      <c r="D85" s="66" t="s">
         <v>560</v>
       </c>
       <c r="E85" s="28" t="s">
@@ -9575,7 +9575,7 @@
       <c r="C87" s="28" t="s">
         <v>518</v>
       </c>
-      <c r="D87" s="76" t="s">
+      <c r="D87" s="66" t="s">
         <v>562</v>
       </c>
       <c r="E87" s="28" t="s">
@@ -9615,7 +9615,7 @@
       <c r="C89" s="28" t="s">
         <v>520</v>
       </c>
-      <c r="D89" s="77" t="s">
+      <c r="D89" s="67" t="s">
         <v>564</v>
       </c>
       <c r="E89" s="28" t="s">
@@ -10340,7 +10340,7 @@
     <row r="155" spans="2:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B155" s="28"/>
       <c r="C155" s="64" t="s">
-        <v>282</v>
+        <v>565</v>
       </c>
       <c r="D155" s="28"/>
       <c r="E155" s="28" t="s">
@@ -10383,10 +10383,10 @@
     </row>
     <row r="160" spans="2:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="161" spans="2:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C161" s="71" t="s">
+      <c r="C161" s="73" t="s">
         <v>540</v>
       </c>
-      <c r="D161" s="71"/>
+      <c r="D161" s="73"/>
     </row>
     <row r="162" spans="2:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="163" spans="2:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>